<commit_message>
boton de excel ya funciona... otra vez, y mas canciones por parte de renko
</commit_message>
<xml_diff>
--- a/FMQ Template.xlsx
+++ b/FMQ Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Youtube Links</t>
   </si>
@@ -57,6 +57,30 @@
   </si>
   <si>
     <t>FMQ Template</t>
+  </si>
+  <si>
+    <t>https://youtu.be/XsDnEXOzxzg?t=32</t>
+  </si>
+  <si>
+    <t>I wanna GNU;I Wanna Kill The Kamilia 2;I wanna be the Shiny spark!!</t>
+  </si>
+  <si>
+    <t>I Wanna Be The Medley</t>
+  </si>
+  <si>
+    <t>hapi⇒</t>
+  </si>
+  <si>
+    <t>https://youtu.be/8sgycukafqQ?t=22</t>
+  </si>
+  <si>
+    <t>ChatGPT Needle</t>
+  </si>
+  <si>
+    <t>What I've Done</t>
+  </si>
+  <si>
+    <t>Linkin Park</t>
   </si>
 </sst>
 </file>
@@ -149,15 +173,6 @@
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -168,6 +183,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -480,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.5703125" customWidth="1"/>
@@ -490,32 +514,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
     </row>
     <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="5" t="s">
         <v>3</v>
       </c>
     </row>
@@ -545,6 +569,34 @@
       </c>
       <c r="D5" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -555,8 +607,10 @@
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1"/>
     <hyperlink ref="A5" r:id="rId2"/>
+    <hyperlink ref="A6" r:id="rId3"/>
+    <hyperlink ref="A7" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Un nuevo sistema para las canciones borradas
</commit_message>
<xml_diff>
--- a/FMQ Template.xlsx
+++ b/FMQ Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Youtube Links</t>
   </si>
@@ -81,6 +81,12 @@
   </si>
   <si>
     <t>Linkin Park</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>OK</t>
   </si>
 </sst>
 </file>
@@ -119,7 +125,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -153,6 +159,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -191,7 +203,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -199,7 +211,74 @@
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <colors>
     <mruColors>
@@ -504,32 +583,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.5703125" customWidth="1"/>
     <col min="2" max="2" width="58.42578125" customWidth="1"/>
     <col min="3" max="3" width="40.85546875" customWidth="1"/>
     <col min="4" max="4" width="39.140625" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
-    <row r="2" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
     </row>
-    <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -542,8 +624,11 @@
       <c r="D3" s="5" t="s">
         <v>3</v>
       </c>
+      <c r="E3" s="8" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -556,8 +641,11 @@
       <c r="D4" t="s">
         <v>7</v>
       </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -570,8 +658,11 @@
       <c r="D5" t="s">
         <v>11</v>
       </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -584,8 +675,11 @@
       <c r="D6" t="s">
         <v>17</v>
       </c>
+      <c r="E6" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
@@ -597,13 +691,29 @@
       </c>
       <c r="D7" t="s">
         <v>21</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
+  <conditionalFormatting sqref="A4:D1000 E4:E7">
+    <cfRule type="expression" priority="2">
+      <formula>$E4="OK"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$E4="Down"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E7">
+      <formula1>"OK,Down"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1"/>
     <hyperlink ref="A5" r:id="rId2"/>

</xml_diff>

<commit_message>
nuevas canciones, y la opcion NSFW añadido
</commit_message>
<xml_diff>
--- a/FMQ Template.xlsx
+++ b/FMQ Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
   <si>
     <t>Youtube Links</t>
   </si>
@@ -87,6 +87,21 @@
   </si>
   <si>
     <t>OK</t>
+  </si>
+  <si>
+    <t>https://youtu.be/02vDkMEdIkY?t=50</t>
+  </si>
+  <si>
+    <t>I Wanna Kill the 2sweepor</t>
+  </si>
+  <si>
+    <t>Scatman's World</t>
+  </si>
+  <si>
+    <t>Scatman John</t>
+  </si>
+  <si>
+    <t>NSFW</t>
   </si>
 </sst>
 </file>
@@ -211,7 +226,54 @@
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -227,6 +289,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF99FF"/>
       <color rgb="FFCCFFCC"/>
     </mruColors>
   </colors>
@@ -528,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.5703125" customWidth="1"/>
@@ -641,22 +704,42 @@
         <v>23</v>
       </c>
     </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A4:D1000 E4:E7">
-    <cfRule type="expression" priority="2">
+  <conditionalFormatting sqref="A4:D1000 E4:E8">
+    <cfRule type="expression" priority="3">
       <formula>$E4="OK"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$E4="Down"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>$E4="NSFW"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E7">
-      <formula1>"OK,Down"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E8">
+      <formula1>"OK,Down,NSFW"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -664,8 +747,9 @@
     <hyperlink ref="A5" r:id="rId2"/>
     <hyperlink ref="A6" r:id="rId3"/>
     <hyperlink ref="A7" r:id="rId4"/>
+    <hyperlink ref="A8" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>